<commit_message>
test: update selenium test report - 54/54 tests passing
</commit_message>
<xml_diff>
--- a/tests/report/selenium-test-results.xlsx
+++ b/tests/report/selenium-test-results.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="144">
   <si>
     <t>Test ID</t>
   </si>
@@ -43,7 +43,7 @@
     <t>Vite build configured</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:16.064Z</t>
+    <t>2026-06-13T08:19:11.417Z</t>
   </si>
   <si>
     <t>Preview works</t>
@@ -52,7 +52,7 @@
     <t>Vite preview available</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:16.065Z</t>
+    <t>2026-06-13T08:19:11.418Z</t>
   </si>
   <si>
     <t>HTTPS backend</t>
@@ -67,7 +67,7 @@
     <t>Home page rendered</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:19.067Z</t>
+    <t>2026-06-13T08:19:14.732Z</t>
   </si>
   <si>
     <t>UI/UX</t>
@@ -79,7 +79,7 @@
     <t>Found 1 headings</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:19.080Z</t>
+    <t>2026-06-13T08:19:14.752Z</t>
   </si>
   <si>
     <t>Features render</t>
@@ -88,7 +88,7 @@
     <t>Found 10 features</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:19.092Z</t>
+    <t>2026-06-13T08:19:14.772Z</t>
   </si>
   <si>
     <t>CTAs visible</t>
@@ -97,7 +97,7 @@
     <t>Found 2 buttons</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:19.102Z</t>
+    <t>2026-06-13T08:19:14.790Z</t>
   </si>
   <si>
     <t>Hero CTAs</t>
@@ -106,7 +106,7 @@
     <t>Found 2 hero actions</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:19.116Z</t>
+    <t>2026-06-13T08:19:14.808Z</t>
   </si>
   <si>
     <t>Functional</t>
@@ -118,7 +118,7 @@
     <t>Home loads</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:19.275Z</t>
+    <t>2026-06-13T08:19:15.049Z</t>
   </si>
   <si>
     <t>Dashboard route</t>
@@ -133,16 +133,16 @@
     <t>Found 3 nav items</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:19.345Z</t>
+    <t>2026-06-13T08:19:15.512Z</t>
   </si>
   <si>
     <t>Dashboard cards</t>
   </si>
   <si>
-    <t>Found 16 cards</t>
-  </si>
-  <si>
-    <t>2026-06-12T08:48:19.372Z</t>
+    <t>Found 19 cards</t>
+  </si>
+  <si>
+    <t>2026-06-13T08:19:15.531Z</t>
   </si>
   <si>
     <t>Jobs route</t>
@@ -151,7 +151,7 @@
     <t>Jobs page loaded</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:19.483Z</t>
+    <t>2026-06-13T08:19:15.765Z</t>
   </si>
   <si>
     <t>Search input</t>
@@ -160,7 +160,7 @@
     <t>Search field found</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:19.869Z</t>
+    <t>2026-06-13T08:19:16.081Z</t>
   </si>
   <si>
     <t>Filters visible</t>
@@ -169,7 +169,7 @@
     <t>Found 2 filters</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:19.880Z</t>
+    <t>2026-06-13T08:19:16.096Z</t>
   </si>
   <si>
     <t>Search works</t>
@@ -178,25 +178,25 @@
     <t>Query entered</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:20.899Z</t>
+    <t>2026-06-13T08:19:17.238Z</t>
   </si>
   <si>
     <t>Job grid</t>
   </si>
   <si>
-    <t>Found 6 jobs</t>
-  </si>
-  <si>
-    <t>2026-06-12T08:48:20.915Z</t>
+    <t>Found 5 jobs</t>
+  </si>
+  <si>
+    <t>2026-06-13T08:19:17.262Z</t>
   </si>
   <si>
     <t>Apply buttons</t>
   </si>
   <si>
-    <t>Found 6 buttons</t>
-  </si>
-  <si>
-    <t>2026-06-12T08:48:20.925Z</t>
+    <t>Found 5 buttons</t>
+  </si>
+  <si>
+    <t>2026-06-13T08:19:17.276Z</t>
   </si>
   <si>
     <t>Validation</t>
@@ -208,7 +208,7 @@
     <t>Search cleared</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:20.946Z</t>
+    <t>2026-06-13T08:19:17.311Z</t>
   </si>
   <si>
     <t>No results</t>
@@ -217,7 +217,7 @@
     <t>0 items</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:22.129Z</t>
+    <t>2026-06-13T08:19:18.644Z</t>
   </si>
   <si>
     <t>Analytics route</t>
@@ -226,7 +226,7 @@
     <t>Analytics loaded</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:22.202Z</t>
+    <t>2026-06-13T08:19:18.724Z</t>
   </si>
   <si>
     <t>Mobile layout</t>
@@ -235,7 +235,7 @@
     <t>Resized to mobile</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:23.774Z</t>
+    <t>2026-06-13T08:19:20.299Z</t>
   </si>
   <si>
     <t>Desktop layout</t>
@@ -244,7 +244,7 @@
     <t>Resized back to desktop</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:24.717Z</t>
+    <t>2026-06-13T08:19:21.138Z</t>
   </si>
   <si>
     <t>API works</t>
@@ -253,7 +253,7 @@
     <t>100 jobs returned</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:25.300Z</t>
+    <t>2026-06-13T08:19:21.983Z</t>
   </si>
   <si>
     <t>Navigation</t>
@@ -268,7 +268,7 @@
     <t>Page refresh succeeds</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:25.865Z</t>
+    <t>2026-06-13T08:19:22.316Z</t>
   </si>
   <si>
     <t>SPA routing</t>
@@ -277,7 +277,7 @@
     <t>Client-side routing</t>
   </si>
   <si>
-    <t>2026-06-12T08:48:26.866Z</t>
+    <t>2026-06-13T08:19:23.320Z</t>
   </si>
   <si>
     <t>Static ready</t>
@@ -299,9 +299,6 @@
   </si>
   <si>
     <t>Keyboard support</t>
-  </si>
-  <si>
-    <t>2026-06-12T08:48:26.867Z</t>
   </si>
   <si>
     <t>Contrast good</t>
@@ -1450,7 +1447,7 @@
         <v>95</v>
       </c>
       <c r="F31" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1461,16 +1458,16 @@
         <v>91</v>
       </c>
       <c r="C32" t="s">
+        <v>96</v>
+      </c>
+      <c r="D32" t="s">
+        <v>8</v>
+      </c>
+      <c r="E32" t="s">
         <v>97</v>
       </c>
-      <c r="D32" t="s">
-        <v>8</v>
-      </c>
-      <c r="E32" t="s">
-        <v>98</v>
-      </c>
       <c r="F32" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1478,19 +1475,19 @@
         <v>71</v>
       </c>
       <c r="B33" t="s">
+        <v>98</v>
+      </c>
+      <c r="C33" t="s">
         <v>99</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
+        <v>8</v>
+      </c>
+      <c r="E33" t="s">
         <v>100</v>
       </c>
-      <c r="D33" t="s">
-        <v>8</v>
-      </c>
-      <c r="E33" t="s">
-        <v>101</v>
-      </c>
       <c r="F33" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1498,19 +1495,19 @@
         <v>73</v>
       </c>
       <c r="B34" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C34" t="s">
+        <v>101</v>
+      </c>
+      <c r="D34" t="s">
+        <v>8</v>
+      </c>
+      <c r="E34" t="s">
         <v>102</v>
       </c>
-      <c r="D34" t="s">
-        <v>8</v>
-      </c>
-      <c r="E34" t="s">
-        <v>103</v>
-      </c>
       <c r="F34" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -1518,19 +1515,19 @@
         <v>75</v>
       </c>
       <c r="B35" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C35" t="s">
+        <v>103</v>
+      </c>
+      <c r="D35" t="s">
+        <v>8</v>
+      </c>
+      <c r="E35" t="s">
         <v>104</v>
       </c>
-      <c r="D35" t="s">
-        <v>8</v>
-      </c>
-      <c r="E35" t="s">
-        <v>105</v>
-      </c>
       <c r="F35" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -1538,19 +1535,19 @@
         <v>76</v>
       </c>
       <c r="B36" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C36" t="s">
+        <v>105</v>
+      </c>
+      <c r="D36" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36" t="s">
         <v>106</v>
       </c>
-      <c r="D36" t="s">
-        <v>8</v>
-      </c>
-      <c r="E36" t="s">
-        <v>107</v>
-      </c>
       <c r="F36" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -1561,16 +1558,16 @@
         <v>62</v>
       </c>
       <c r="C37" t="s">
+        <v>107</v>
+      </c>
+      <c r="D37" t="s">
+        <v>8</v>
+      </c>
+      <c r="E37" t="s">
         <v>108</v>
       </c>
-      <c r="D37" t="s">
-        <v>8</v>
-      </c>
-      <c r="E37" t="s">
-        <v>109</v>
-      </c>
       <c r="F37" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -1581,16 +1578,16 @@
         <v>62</v>
       </c>
       <c r="C38" t="s">
+        <v>109</v>
+      </c>
+      <c r="D38" t="s">
+        <v>8</v>
+      </c>
+      <c r="E38" t="s">
         <v>110</v>
       </c>
-      <c r="D38" t="s">
-        <v>8</v>
-      </c>
-      <c r="E38" t="s">
-        <v>111</v>
-      </c>
       <c r="F38" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -1601,16 +1598,16 @@
         <v>62</v>
       </c>
       <c r="C39" t="s">
+        <v>111</v>
+      </c>
+      <c r="D39" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39" t="s">
         <v>112</v>
       </c>
-      <c r="D39" t="s">
-        <v>8</v>
-      </c>
-      <c r="E39" t="s">
-        <v>113</v>
-      </c>
       <c r="F39" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -1621,16 +1618,16 @@
         <v>62</v>
       </c>
       <c r="C40" t="s">
+        <v>113</v>
+      </c>
+      <c r="D40" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40" t="s">
         <v>114</v>
       </c>
-      <c r="D40" t="s">
-        <v>8</v>
-      </c>
-      <c r="E40" t="s">
-        <v>115</v>
-      </c>
       <c r="F40" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -1641,16 +1638,16 @@
         <v>62</v>
       </c>
       <c r="C41" t="s">
+        <v>115</v>
+      </c>
+      <c r="D41" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41" t="s">
         <v>116</v>
       </c>
-      <c r="D41" t="s">
-        <v>8</v>
-      </c>
-      <c r="E41" t="s">
-        <v>117</v>
-      </c>
       <c r="F41" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -1661,16 +1658,16 @@
         <v>62</v>
       </c>
       <c r="C42" t="s">
+        <v>117</v>
+      </c>
+      <c r="D42" t="s">
+        <v>8</v>
+      </c>
+      <c r="E42" t="s">
         <v>118</v>
       </c>
-      <c r="D42" t="s">
-        <v>8</v>
-      </c>
-      <c r="E42" t="s">
-        <v>119</v>
-      </c>
       <c r="F42" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -1681,16 +1678,16 @@
         <v>19</v>
       </c>
       <c r="C43" t="s">
+        <v>119</v>
+      </c>
+      <c r="D43" t="s">
+        <v>8</v>
+      </c>
+      <c r="E43" t="s">
         <v>120</v>
       </c>
-      <c r="D43" t="s">
-        <v>8</v>
-      </c>
-      <c r="E43" t="s">
-        <v>121</v>
-      </c>
       <c r="F43" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -1701,16 +1698,16 @@
         <v>19</v>
       </c>
       <c r="C44" t="s">
+        <v>121</v>
+      </c>
+      <c r="D44" t="s">
+        <v>8</v>
+      </c>
+      <c r="E44" t="s">
         <v>122</v>
       </c>
-      <c r="D44" t="s">
-        <v>8</v>
-      </c>
-      <c r="E44" t="s">
-        <v>123</v>
-      </c>
       <c r="F44" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -1721,16 +1718,16 @@
         <v>19</v>
       </c>
       <c r="C45" t="s">
+        <v>123</v>
+      </c>
+      <c r="D45" t="s">
+        <v>8</v>
+      </c>
+      <c r="E45" t="s">
         <v>124</v>
       </c>
-      <c r="D45" t="s">
-        <v>8</v>
-      </c>
-      <c r="E45" t="s">
-        <v>125</v>
-      </c>
       <c r="F45" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -1741,16 +1738,16 @@
         <v>19</v>
       </c>
       <c r="C46" t="s">
+        <v>125</v>
+      </c>
+      <c r="D46" t="s">
+        <v>8</v>
+      </c>
+      <c r="E46" t="s">
         <v>126</v>
       </c>
-      <c r="D46" t="s">
-        <v>8</v>
-      </c>
-      <c r="E46" t="s">
-        <v>127</v>
-      </c>
       <c r="F46" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -1761,16 +1758,16 @@
         <v>19</v>
       </c>
       <c r="C47" t="s">
+        <v>127</v>
+      </c>
+      <c r="D47" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" t="s">
         <v>128</v>
       </c>
-      <c r="D47" t="s">
-        <v>8</v>
-      </c>
-      <c r="E47" t="s">
-        <v>129</v>
-      </c>
       <c r="F47" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -1781,16 +1778,16 @@
         <v>19</v>
       </c>
       <c r="C48" t="s">
+        <v>129</v>
+      </c>
+      <c r="D48" t="s">
+        <v>8</v>
+      </c>
+      <c r="E48" t="s">
         <v>130</v>
       </c>
-      <c r="D48" t="s">
-        <v>8</v>
-      </c>
-      <c r="E48" t="s">
-        <v>131</v>
-      </c>
       <c r="F48" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -1801,16 +1798,16 @@
         <v>32</v>
       </c>
       <c r="C49" t="s">
+        <v>131</v>
+      </c>
+      <c r="D49" t="s">
+        <v>8</v>
+      </c>
+      <c r="E49" t="s">
         <v>132</v>
       </c>
-      <c r="D49" t="s">
-        <v>8</v>
-      </c>
-      <c r="E49" t="s">
-        <v>133</v>
-      </c>
       <c r="F49" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -1821,16 +1818,16 @@
         <v>32</v>
       </c>
       <c r="C50" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D50" t="s">
         <v>8</v>
       </c>
       <c r="E50" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F50" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -1841,16 +1838,16 @@
         <v>32</v>
       </c>
       <c r="C51" t="s">
+        <v>134</v>
+      </c>
+      <c r="D51" t="s">
+        <v>8</v>
+      </c>
+      <c r="E51" t="s">
         <v>135</v>
       </c>
-      <c r="D51" t="s">
-        <v>8</v>
-      </c>
-      <c r="E51" t="s">
-        <v>136</v>
-      </c>
       <c r="F51" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -1861,16 +1858,16 @@
         <v>32</v>
       </c>
       <c r="C52" t="s">
+        <v>136</v>
+      </c>
+      <c r="D52" t="s">
+        <v>8</v>
+      </c>
+      <c r="E52" t="s">
         <v>137</v>
       </c>
-      <c r="D52" t="s">
-        <v>8</v>
-      </c>
-      <c r="E52" t="s">
-        <v>138</v>
-      </c>
       <c r="F52" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -1881,16 +1878,16 @@
         <v>32</v>
       </c>
       <c r="C53" t="s">
+        <v>138</v>
+      </c>
+      <c r="D53" t="s">
+        <v>8</v>
+      </c>
+      <c r="E53" t="s">
         <v>139</v>
       </c>
-      <c r="D53" t="s">
-        <v>8</v>
-      </c>
-      <c r="E53" t="s">
-        <v>140</v>
-      </c>
       <c r="F53" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -1901,16 +1898,16 @@
         <v>32</v>
       </c>
       <c r="C54" t="s">
+        <v>140</v>
+      </c>
+      <c r="D54" t="s">
+        <v>8</v>
+      </c>
+      <c r="E54" t="s">
         <v>141</v>
       </c>
-      <c r="D54" t="s">
-        <v>8</v>
-      </c>
-      <c r="E54" t="s">
-        <v>142</v>
-      </c>
       <c r="F54" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -1921,16 +1918,16 @@
         <v>32</v>
       </c>
       <c r="C55" t="s">
+        <v>142</v>
+      </c>
+      <c r="D55" t="s">
+        <v>8</v>
+      </c>
+      <c r="E55" t="s">
         <v>143</v>
       </c>
-      <c r="D55" t="s">
-        <v>8</v>
-      </c>
-      <c r="E55" t="s">
-        <v>144</v>
-      </c>
       <c r="F55" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test: all 54 selenium tests passing
</commit_message>
<xml_diff>
--- a/tests/report/selenium-test-results.xlsx
+++ b/tests/report/selenium-test-results.xlsx
@@ -43,7 +43,7 @@
     <t>Vite build configured</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:11.417Z</t>
+    <t>2026-06-13T08:46:34.374Z</t>
   </si>
   <si>
     <t>Preview works</t>
@@ -52,7 +52,7 @@
     <t>Vite preview available</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:11.418Z</t>
+    <t>2026-06-13T08:46:34.385Z</t>
   </si>
   <si>
     <t>HTTPS backend</t>
@@ -67,7 +67,7 @@
     <t>Home page rendered</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:14.732Z</t>
+    <t>2026-06-13T08:46:37.228Z</t>
   </si>
   <si>
     <t>UI/UX</t>
@@ -79,7 +79,7 @@
     <t>Found 1 headings</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:14.752Z</t>
+    <t>2026-06-13T08:46:37.255Z</t>
   </si>
   <si>
     <t>Features render</t>
@@ -88,7 +88,7 @@
     <t>Found 10 features</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:14.772Z</t>
+    <t>2026-06-13T08:46:37.279Z</t>
   </si>
   <si>
     <t>CTAs visible</t>
@@ -97,7 +97,7 @@
     <t>Found 2 buttons</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:14.790Z</t>
+    <t>2026-06-13T08:46:37.305Z</t>
   </si>
   <si>
     <t>Hero CTAs</t>
@@ -106,7 +106,7 @@
     <t>Found 2 hero actions</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:14.808Z</t>
+    <t>2026-06-13T08:46:37.327Z</t>
   </si>
   <si>
     <t>Functional</t>
@@ -118,7 +118,7 @@
     <t>Home loads</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:15.049Z</t>
+    <t>2026-06-13T08:46:37.642Z</t>
   </si>
   <si>
     <t>Dashboard route</t>
@@ -133,16 +133,16 @@
     <t>Found 3 nav items</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:15.512Z</t>
+    <t>2026-06-13T08:46:38.259Z</t>
   </si>
   <si>
     <t>Dashboard cards</t>
   </si>
   <si>
-    <t>Found 19 cards</t>
-  </si>
-  <si>
-    <t>2026-06-13T08:19:15.531Z</t>
+    <t>Found 20 cards</t>
+  </si>
+  <si>
+    <t>2026-06-13T08:46:38.286Z</t>
   </si>
   <si>
     <t>Jobs route</t>
@@ -151,7 +151,7 @@
     <t>Jobs page loaded</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:15.765Z</t>
+    <t>2026-06-13T08:46:38.765Z</t>
   </si>
   <si>
     <t>Search input</t>
@@ -160,7 +160,7 @@
     <t>Search field found</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:16.081Z</t>
+    <t>2026-06-13T08:46:39.175Z</t>
   </si>
   <si>
     <t>Filters visible</t>
@@ -169,7 +169,7 @@
     <t>Found 2 filters</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:16.096Z</t>
+    <t>2026-06-13T08:46:39.204Z</t>
   </si>
   <si>
     <t>Search works</t>
@@ -178,7 +178,7 @@
     <t>Query entered</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:17.238Z</t>
+    <t>2026-06-13T08:46:40.426Z</t>
   </si>
   <si>
     <t>Job grid</t>
@@ -187,7 +187,7 @@
     <t>Found 5 jobs</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:17.262Z</t>
+    <t>2026-06-13T08:46:40.458Z</t>
   </si>
   <si>
     <t>Apply buttons</t>
@@ -196,7 +196,7 @@
     <t>Found 5 buttons</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:17.276Z</t>
+    <t>2026-06-13T08:46:40.482Z</t>
   </si>
   <si>
     <t>Validation</t>
@@ -208,7 +208,7 @@
     <t>Search cleared</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:17.311Z</t>
+    <t>2026-06-13T08:46:40.526Z</t>
   </si>
   <si>
     <t>No results</t>
@@ -217,7 +217,7 @@
     <t>0 items</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:18.644Z</t>
+    <t>2026-06-13T08:46:41.952Z</t>
   </si>
   <si>
     <t>Analytics route</t>
@@ -226,7 +226,7 @@
     <t>Analytics loaded</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:18.724Z</t>
+    <t>2026-06-13T08:46:42.062Z</t>
   </si>
   <si>
     <t>Mobile layout</t>
@@ -235,7 +235,7 @@
     <t>Resized to mobile</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:20.299Z</t>
+    <t>2026-06-13T08:46:43.675Z</t>
   </si>
   <si>
     <t>Desktop layout</t>
@@ -244,7 +244,7 @@
     <t>Resized back to desktop</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:21.138Z</t>
+    <t>2026-06-13T08:46:44.824Z</t>
   </si>
   <si>
     <t>API works</t>
@@ -253,7 +253,7 @@
     <t>100 jobs returned</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:21.983Z</t>
+    <t>2026-06-13T08:46:46.203Z</t>
   </si>
   <si>
     <t>Navigation</t>
@@ -268,7 +268,7 @@
     <t>Page refresh succeeds</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:22.316Z</t>
+    <t>2026-06-13T08:46:46.643Z</t>
   </si>
   <si>
     <t>SPA routing</t>
@@ -277,7 +277,7 @@
     <t>Client-side routing</t>
   </si>
   <si>
-    <t>2026-06-13T08:19:23.320Z</t>
+    <t>2026-06-13T08:46:47.652Z</t>
   </si>
   <si>
     <t>Static ready</t>

</xml_diff>

<commit_message>
fix: resolve E2E Selenium tests crash and run reports workflow on all branch pushes
</commit_message>
<xml_diff>
--- a/tests/report/selenium-test-results.xlsx
+++ b/tests/report/selenium-test-results.xlsx
@@ -43,7 +43,7 @@
     <t>Vite build configured</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:34.374Z</t>
+    <t>2026-06-13T09:06:05.128Z</t>
   </si>
   <si>
     <t>Preview works</t>
@@ -52,7 +52,7 @@
     <t>Vite preview available</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:34.385Z</t>
+    <t>2026-06-13T09:06:05.142Z</t>
   </si>
   <si>
     <t>HTTPS backend</t>
@@ -67,7 +67,7 @@
     <t>Home page rendered</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:37.228Z</t>
+    <t>2026-06-13T09:06:07.726Z</t>
   </si>
   <si>
     <t>UI/UX</t>
@@ -79,7 +79,7 @@
     <t>Found 1 headings</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:37.255Z</t>
+    <t>2026-06-13T09:06:07.743Z</t>
   </si>
   <si>
     <t>Features render</t>
@@ -88,7 +88,7 @@
     <t>Found 10 features</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:37.279Z</t>
+    <t>2026-06-13T09:06:07.763Z</t>
   </si>
   <si>
     <t>CTAs visible</t>
@@ -97,7 +97,7 @@
     <t>Found 2 buttons</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:37.305Z</t>
+    <t>2026-06-13T09:06:07.799Z</t>
   </si>
   <si>
     <t>Hero CTAs</t>
@@ -106,7 +106,7 @@
     <t>Found 2 hero actions</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:37.327Z</t>
+    <t>2026-06-13T09:06:07.821Z</t>
   </si>
   <si>
     <t>Functional</t>
@@ -118,7 +118,7 @@
     <t>Home loads</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:37.642Z</t>
+    <t>2026-06-13T09:06:08.067Z</t>
   </si>
   <si>
     <t>Dashboard route</t>
@@ -133,7 +133,7 @@
     <t>Found 3 nav items</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:38.259Z</t>
+    <t>2026-06-13T09:06:08.519Z</t>
   </si>
   <si>
     <t>Dashboard cards</t>
@@ -142,7 +142,7 @@
     <t>Found 20 cards</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:38.286Z</t>
+    <t>2026-06-13T09:06:08.540Z</t>
   </si>
   <si>
     <t>Jobs route</t>
@@ -151,7 +151,7 @@
     <t>Jobs page loaded</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:38.765Z</t>
+    <t>2026-06-13T09:06:08.807Z</t>
   </si>
   <si>
     <t>Search input</t>
@@ -160,7 +160,7 @@
     <t>Search field found</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:39.175Z</t>
+    <t>2026-06-13T09:06:09.089Z</t>
   </si>
   <si>
     <t>Filters visible</t>
@@ -169,7 +169,7 @@
     <t>Found 2 filters</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:39.204Z</t>
+    <t>2026-06-13T09:06:09.102Z</t>
   </si>
   <si>
     <t>Search works</t>
@@ -178,7 +178,7 @@
     <t>Query entered</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:40.426Z</t>
+    <t>2026-06-13T09:06:10.394Z</t>
   </si>
   <si>
     <t>Job grid</t>
@@ -187,7 +187,7 @@
     <t>Found 5 jobs</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:40.458Z</t>
+    <t>2026-06-13T09:06:10.419Z</t>
   </si>
   <si>
     <t>Apply buttons</t>
@@ -196,7 +196,7 @@
     <t>Found 5 buttons</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:40.482Z</t>
+    <t>2026-06-13T09:06:10.433Z</t>
   </si>
   <si>
     <t>Validation</t>
@@ -208,7 +208,7 @@
     <t>Search cleared</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:40.526Z</t>
+    <t>2026-06-13T09:06:10.466Z</t>
   </si>
   <si>
     <t>No results</t>
@@ -217,7 +217,7 @@
     <t>0 items</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:41.952Z</t>
+    <t>2026-06-13T09:06:11.842Z</t>
   </si>
   <si>
     <t>Analytics route</t>
@@ -226,7 +226,7 @@
     <t>Analytics loaded</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:42.062Z</t>
+    <t>2026-06-13T09:06:11.956Z</t>
   </si>
   <si>
     <t>Mobile layout</t>
@@ -235,7 +235,7 @@
     <t>Resized to mobile</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:43.675Z</t>
+    <t>2026-06-13T09:06:13.568Z</t>
   </si>
   <si>
     <t>Desktop layout</t>
@@ -244,7 +244,7 @@
     <t>Resized back to desktop</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:44.824Z</t>
+    <t>2026-06-13T09:06:14.757Z</t>
   </si>
   <si>
     <t>API works</t>
@@ -253,7 +253,7 @@
     <t>100 jobs returned</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:46.203Z</t>
+    <t>2026-06-13T09:06:15.182Z</t>
   </si>
   <si>
     <t>Navigation</t>
@@ -268,7 +268,7 @@
     <t>Page refresh succeeds</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:46.643Z</t>
+    <t>2026-06-13T09:06:16.120Z</t>
   </si>
   <si>
     <t>SPA routing</t>
@@ -277,7 +277,7 @@
     <t>Client-side routing</t>
   </si>
   <si>
-    <t>2026-06-13T08:46:47.652Z</t>
+    <t>2026-06-13T09:06:17.121Z</t>
   </si>
   <si>
     <t>Static ready</t>

</xml_diff>

<commit_message>
fix: resolve E2E tests timeout hang and Node 20 deprecation warnings
</commit_message>
<xml_diff>
--- a/tests/report/selenium-test-results.xlsx
+++ b/tests/report/selenium-test-results.xlsx
@@ -43,7 +43,7 @@
     <t>Vite build configured</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:05.128Z</t>
+    <t>2026-06-15T05:10:42.355Z</t>
   </si>
   <si>
     <t>Preview works</t>
@@ -52,7 +52,7 @@
     <t>Vite preview available</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:05.142Z</t>
+    <t>2026-06-15T05:10:42.356Z</t>
   </si>
   <si>
     <t>HTTPS backend</t>
@@ -67,7 +67,7 @@
     <t>Home page rendered</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:07.726Z</t>
+    <t>2026-06-15T05:10:55.691Z</t>
   </si>
   <si>
     <t>UI/UX</t>
@@ -79,7 +79,7 @@
     <t>Found 1 headings</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:07.743Z</t>
+    <t>2026-06-15T05:10:55.702Z</t>
   </si>
   <si>
     <t>Features render</t>
@@ -88,7 +88,7 @@
     <t>Found 10 features</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:07.763Z</t>
+    <t>2026-06-15T05:10:55.713Z</t>
   </si>
   <si>
     <t>CTAs visible</t>
@@ -97,7 +97,7 @@
     <t>Found 2 buttons</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:07.799Z</t>
+    <t>2026-06-15T05:10:55.720Z</t>
   </si>
   <si>
     <t>Hero CTAs</t>
@@ -106,7 +106,7 @@
     <t>Found 2 hero actions</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:07.821Z</t>
+    <t>2026-06-15T05:10:55.731Z</t>
   </si>
   <si>
     <t>Functional</t>
@@ -118,7 +118,7 @@
     <t>Home loads</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:08.067Z</t>
+    <t>2026-06-15T05:10:55.834Z</t>
   </si>
   <si>
     <t>Dashboard route</t>
@@ -133,16 +133,16 @@
     <t>Found 3 nav items</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:08.519Z</t>
+    <t>2026-06-15T05:10:56.084Z</t>
   </si>
   <si>
     <t>Dashboard cards</t>
   </si>
   <si>
-    <t>Found 20 cards</t>
-  </si>
-  <si>
-    <t>2026-06-13T09:06:08.540Z</t>
+    <t>Found 16 cards</t>
+  </si>
+  <si>
+    <t>2026-06-15T05:10:56.092Z</t>
   </si>
   <si>
     <t>Jobs route</t>
@@ -151,7 +151,7 @@
     <t>Jobs page loaded</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:08.807Z</t>
+    <t>2026-06-15T05:10:56.149Z</t>
   </si>
   <si>
     <t>Search input</t>
@@ -160,7 +160,7 @@
     <t>Search field found</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:09.089Z</t>
+    <t>2026-06-15T05:10:57.612Z</t>
   </si>
   <si>
     <t>Filters visible</t>
@@ -169,7 +169,7 @@
     <t>Found 2 filters</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:09.102Z</t>
+    <t>2026-06-15T05:10:57.621Z</t>
   </si>
   <si>
     <t>Search works</t>
@@ -178,7 +178,7 @@
     <t>Query entered</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:10.394Z</t>
+    <t>2026-06-15T05:10:58.638Z</t>
   </si>
   <si>
     <t>Job grid</t>
@@ -187,7 +187,7 @@
     <t>Found 5 jobs</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:10.419Z</t>
+    <t>2026-06-15T05:10:58.648Z</t>
   </si>
   <si>
     <t>Apply buttons</t>
@@ -196,7 +196,7 @@
     <t>Found 5 buttons</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:10.433Z</t>
+    <t>2026-06-15T05:10:58.655Z</t>
   </si>
   <si>
     <t>Validation</t>
@@ -208,7 +208,7 @@
     <t>Search cleared</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:10.466Z</t>
+    <t>2026-06-15T05:10:58.671Z</t>
   </si>
   <si>
     <t>No results</t>
@@ -217,7 +217,7 @@
     <t>0 items</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:11.842Z</t>
+    <t>2026-06-15T05:10:59.741Z</t>
   </si>
   <si>
     <t>Analytics route</t>
@@ -226,7 +226,7 @@
     <t>Analytics loaded</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:11.956Z</t>
+    <t>2026-06-15T05:10:59.962Z</t>
   </si>
   <si>
     <t>Mobile layout</t>
@@ -235,7 +235,7 @@
     <t>Resized to mobile</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:13.568Z</t>
+    <t>2026-06-15T05:11:01.536Z</t>
   </si>
   <si>
     <t>Desktop layout</t>
@@ -244,7 +244,7 @@
     <t>Resized back to desktop</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:14.757Z</t>
+    <t>2026-06-15T05:11:02.368Z</t>
   </si>
   <si>
     <t>API works</t>
@@ -253,7 +253,7 @@
     <t>100 jobs returned</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:15.182Z</t>
+    <t>2026-06-15T05:11:03.272Z</t>
   </si>
   <si>
     <t>Navigation</t>
@@ -268,7 +268,7 @@
     <t>Page refresh succeeds</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:16.120Z</t>
+    <t>2026-06-15T05:11:03.462Z</t>
   </si>
   <si>
     <t>SPA routing</t>
@@ -277,7 +277,7 @@
     <t>Client-side routing</t>
   </si>
   <si>
-    <t>2026-06-13T09:06:17.121Z</t>
+    <t>2026-06-15T05:11:04.462Z</t>
   </si>
   <si>
     <t>Static ready</t>

</xml_diff>